<commit_message>
docs: update server address and jury workbook download
</commit_message>
<xml_diff>
--- a/docs/jury/platform-access.xlsx
+++ b/docs/jury/platform-access.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10500"/>
+    <workbookView windowWidth="23040" windowHeight="9900"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,25 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
+  <si>
+    <t>Название команды:</t>
+  </si>
+  <si>
+    <t>Seg_Fault</t>
+  </si>
+  <si>
+    <t>Адрес платформы:</t>
+  </si>
+  <si>
+    <t>https://honey-forge-seg-fault.ru/</t>
+  </si>
+  <si>
+    <t>Перед заходом на платформу пишем (локально на своём ПК) в конце конфига "hosts" ip-адрес и домен нашего сервера:</t>
+  </si>
+  <si>
+    <t>103.74.94.55  https://honey-forge-seg-fault.ru</t>
+  </si>
   <si>
     <t>Эксперты/Жюри</t>
   </si>
@@ -81,12 +99,6 @@
   </si>
   <si>
     <t>user5@Madrigal-squad.ru</t>
-  </si>
-  <si>
-    <t>Гит-репозитории:</t>
-  </si>
-  <si>
-    <t>https://github.com/Cricko7/honey-forge</t>
   </si>
 </sst>
 </file>
@@ -99,9 +111,47 @@
     <numFmt numFmtId="176" formatCode="_-* #,##0.00\ &quot;₽&quot;_-;\-* #,##0.00\ &quot;₽&quot;_-;_-* &quot;-&quot;??\ &quot;₽&quot;_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-* #,##0\ &quot;₽&quot;_-;\-* #,##0\ &quot;₽&quot;_-;_-* &quot;-&quot;\ &quot;₽&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -116,21 +166,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <i/>
       <sz val="12"/>
       <color theme="1"/>
@@ -142,14 +177,6 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -489,6 +516,15 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -496,21 +532,6 @@
         <color auto="1"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -557,6 +578,21 @@
       <right style="thin">
         <color auto="1"/>
       </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color auto="1"/>
@@ -567,7 +603,9 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -577,17 +615,6 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -743,202 +770,238 @@
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="6" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1465,241 +1528,278 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="C3:H19"/>
+  <dimension ref="C1:H22"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="40.4444444444444" customWidth="1"/>
-    <col min="8" max="8" width="30.1111111111111" customWidth="1"/>
+    <col min="4" max="4" width="25.8888888888889" customWidth="1"/>
+    <col min="5" max="5" width="33.5555555555556" customWidth="1"/>
+    <col min="8" max="8" width="21.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" ht="52" customHeight="1" spans="3:8">
-      <c r="C3" s="1" t="s">
+    <row r="1" ht="33" customHeight="1"/>
+    <row r="2" ht="28" customHeight="1" spans="3:8">
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5"/>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="3:8">
-      <c r="C4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="4" t="s">
+    <row r="3" ht="26" customHeight="1" spans="3:8">
+      <c r="C3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
     </row>
-    <row r="5" ht="34" customHeight="1" spans="3:8">
-      <c r="C5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="8" t="s">
+    <row r="4" ht="65" customHeight="1" spans="3:8">
+      <c r="C4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="10"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
-    <row r="6" ht="26" customHeight="1" spans="3:8">
-      <c r="C6" s="11" t="s">
+    <row r="5" ht="23" customHeight="1" spans="3:8">
+      <c r="C5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13" t="s">
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="31" customHeight="1" spans="3:8">
+      <c r="C8" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
     </row>
-    <row r="7" ht="42" customHeight="1" spans="3:8">
-      <c r="C7" s="17" t="s">
+    <row r="9" ht="46" customHeight="1" spans="3:8">
+      <c r="C9" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="18"/>
-      <c r="E7" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="18" t="s">
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-    </row>
-    <row r="8" ht="42" customHeight="1" spans="3:8">
-      <c r="C8" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="18"/>
-      <c r="E8" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-    </row>
-    <row r="9" ht="42" customHeight="1" spans="3:8">
-      <c r="C9" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="18"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="3:8">
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
+    <row r="10" ht="28" customHeight="1" spans="3:8">
+      <c r="C10" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="21"/>
+      <c r="H10" s="22"/>
     </row>
-    <row r="11" ht="48" customHeight="1" spans="3:8">
-      <c r="C11" s="17" t="s">
+    <row r="11" ht="26" customHeight="1" spans="3:8">
+      <c r="C11" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="26"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="28"/>
+    </row>
+    <row r="12" ht="41" customHeight="1" spans="3:8">
+      <c r="C12" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="17" t="s">
+      <c r="D12" s="30"/>
+      <c r="E12" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
+      <c r="F12" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
     </row>
-    <row r="12" ht="43" customHeight="1" spans="3:8">
-      <c r="C12" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
+    <row r="13" ht="45" customHeight="1" spans="3:8">
+      <c r="C13" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="30"/>
+      <c r="E13" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
     </row>
-    <row r="13" ht="44" customHeight="1" spans="3:8">
-      <c r="C13" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
+    <row r="14" ht="41" customHeight="1" spans="3:8">
+      <c r="C14" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="30"/>
+      <c r="E14" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
     </row>
-    <row r="14" ht="55" customHeight="1" spans="3:8">
-      <c r="C14" s="17" t="s">
+    <row r="15" ht="20" customHeight="1" spans="3:8">
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+    </row>
+    <row r="16" ht="42" customHeight="1" spans="3:8">
+      <c r="C16" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="30"/>
+      <c r="E16" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+    </row>
+    <row r="17" ht="39" customHeight="1" spans="3:8">
+      <c r="C17" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="30"/>
+      <c r="E17" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+    </row>
+    <row r="18" ht="41" customHeight="1" spans="3:8">
+      <c r="C18" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="30"/>
+      <c r="E18" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+    </row>
+    <row r="19" ht="40" customHeight="1" spans="3:8">
+      <c r="C19" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="30"/>
+      <c r="E19" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+    </row>
+    <row r="20" ht="39" customHeight="1" spans="3:8">
+      <c r="C20" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="30"/>
+      <c r="E20" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="18"/>
-      <c r="E14" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
     </row>
-    <row r="15" ht="46" customHeight="1" spans="3:8">
-      <c r="C15" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="16" ht="35" customHeight="1"/>
-    <row r="18" spans="3:5">
-      <c r="C18" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-    </row>
-    <row r="19" ht="25" customHeight="1" spans="3:5">
-      <c r="C19" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-    </row>
+    <row r="21" ht="21" customHeight="1"/>
+    <row r="22" ht="16" customHeight="1"/>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="C9:D9"/>
+  <mergeCells count="29">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="C9:E9"/>
     <mergeCell ref="F9:H9"/>
-    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:H11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="F12:H12"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="F13:H13"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="F14:H14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="C15:H15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F10:H11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C7" r:id="rId1" display="admin@Madrigal-squad.ru" tooltip="mailto:admin@Madrigal-squad.ru"/>
-    <hyperlink ref="C8" r:id="rId2" display="syharik3316@Madrigal-squad.ru" tooltip="mailto:syharik3316@Madrigal-squad.ru"/>
-    <hyperlink ref="C9" r:id="rId3" display="kdjirl@Madrigal-squad.ru" tooltip="mailto:kdjirl@Madrigal-squad.ru"/>
-    <hyperlink ref="C11" r:id="rId4" display="user1@Madrigal-squad.ru" tooltip="mailto:user1@Madrigal-squad.ru"/>
-    <hyperlink ref="C12" r:id="rId5" display="user2@Madrigal-squad.ru" tooltip="mailto:user2@Madrigal-squad.ru"/>
-    <hyperlink ref="C13" r:id="rId6" display="user3@Madrigal-squad.ru" tooltip="mailto:user3@Madrigal-squad.ru"/>
-    <hyperlink ref="C14" r:id="rId7" display="user4@Madrigal-squad.ru" tooltip="mailto:user4@Madrigal-squad.ru"/>
-    <hyperlink ref="C15" r:id="rId8" display="user5@Madrigal-squad.ru" tooltip="mailto:user5@Madrigal-squad.ru"/>
-    <hyperlink ref="E9" r:id="rId3" display="kdjirl@Madrigal-squad.ru"/>
-    <hyperlink ref="E11" r:id="rId4" display="user1@Madrigal-squad.ru" tooltip="mailto:user1@Madrigal-squad.ru"/>
-    <hyperlink ref="E12" r:id="rId5" display="user2@Madrigal-squad.ru"/>
-    <hyperlink ref="E13" r:id="rId6" display="user3@Madrigal-squad.ru"/>
-    <hyperlink ref="E14" r:id="rId7" display="user4@Madrigal-squad.ru"/>
-    <hyperlink ref="E15" r:id="rId8" display="user5@Madrigal-squad.ru"/>
-    <hyperlink ref="E8" r:id="rId2" display="syharik3316@Madrigal-squad.ru"/>
-    <hyperlink ref="E7" r:id="rId1" display="admin@Madrigal-squad.ru"/>
-    <hyperlink ref="C19" r:id="rId9" display="https://github.com/Cricko7/honey-forge"/>
+    <hyperlink ref="E3" r:id="rId1" display="https://honey-forge-seg-fault.ru/" tooltip="https://honey-forge-seg-fault.ru/"/>
+    <hyperlink ref="C12" r:id="rId2" display="admin@Madrigal-squad.ru" tooltip="mailto:admin@Madrigal-squad.ru"/>
+    <hyperlink ref="C13" r:id="rId3" display="syharik3316@Madrigal-squad.ru" tooltip="mailto:syharik3316@Madrigal-squad.ru"/>
+    <hyperlink ref="C14" r:id="rId4" display="kdjirl@Madrigal-squad.ru" tooltip="mailto:kdjirl@Madrigal-squad.ru"/>
+    <hyperlink ref="C16" r:id="rId5" display="user1@Madrigal-squad.ru" tooltip="mailto:user1@Madrigal-squad.ru"/>
+    <hyperlink ref="C17" r:id="rId6" display="user2@Madrigal-squad.ru" tooltip="mailto:user2@Madrigal-squad.ru"/>
+    <hyperlink ref="C18" r:id="rId7" display="user3@Madrigal-squad.ru" tooltip="mailto:user3@Madrigal-squad.ru"/>
+    <hyperlink ref="C19" r:id="rId8" display="user4@Madrigal-squad.ru" tooltip="mailto:user4@Madrigal-squad.ru"/>
+    <hyperlink ref="C20" r:id="rId9" display="user5@Madrigal-squad.ru" tooltip="mailto:user5@Madrigal-squad.ru"/>
+    <hyperlink ref="E14" r:id="rId4" display="kdjirl@Madrigal-squad.ru"/>
+    <hyperlink ref="E16" r:id="rId5" display="user1@Madrigal-squad.ru" tooltip="mailto:user1@Madrigal-squad.ru"/>
+    <hyperlink ref="E17" r:id="rId6" display="user2@Madrigal-squad.ru"/>
+    <hyperlink ref="E18" r:id="rId7" display="user3@Madrigal-squad.ru"/>
+    <hyperlink ref="E19" r:id="rId8" display="user4@Madrigal-squad.ru"/>
+    <hyperlink ref="E20" r:id="rId9" display="user5@Madrigal-squad.ru"/>
+    <hyperlink ref="E13" r:id="rId3" display="syharik3316@Madrigal-squad.ru"/>
+    <hyperlink ref="E12" r:id="rId2" display="admin@Madrigal-squad.ru"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>